<commit_message>
Version sent to advisors.
</commit_message>
<xml_diff>
--- a/diagramas/diagrama_Gantt.xlsx
+++ b/diagramas/diagrama_Gantt.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28324"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28429"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Ricardo\Desktop\Tese_mestrado\diagramas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4BCE4E19-1244-4E79-9551-56274FAD60A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8FBB4082-AD08-4265-A554-750B0CC751D4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{9E5D4881-DCE1-478A-8E87-A90D197304B3}"/>
   </bookViews>
@@ -81,13 +81,13 @@
     <t>Duração (semanas)</t>
   </si>
   <si>
-    <t>Conversão dos dados de entrada para o padrão ITC 2019</t>
-  </si>
-  <si>
     <t>Implementação do interpretador dos dados ITC 2019</t>
   </si>
   <si>
     <t>Planeamento da arquitetura</t>
+  </si>
+  <si>
+    <t>Correção de erros</t>
   </si>
 </sst>
 </file>
@@ -132,7 +132,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -143,13 +143,16 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -227,19 +230,19 @@
                   <c:v>Planeamento da arquitetura</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>Conversão dos dados de entrada para o padrão ITC 2019</c:v>
+                  <c:v>Implementação do interpretador dos dados ITC 2019</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>Implementação do interpretador dos dados ITC 2019</c:v>
+                  <c:v>Implementação da base de dados</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>Implementação da base de dados</c:v>
+                  <c:v>Implementação do simulated annealing</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>Implementação do simulated annealing</c:v>
+                  <c:v>Implementação da interface gráfica</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>Implementação da interface gráfica</c:v>
+                  <c:v>Correção de erros</c:v>
                 </c:pt>
                 <c:pt idx="7">
                   <c:v>Avaliação e correção da aplicação</c:v>
@@ -260,22 +263,22 @@
                   <c:v>45717</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>45717</c:v>
+                  <c:v>45745</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>45722</c:v>
+                  <c:v>45763</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>45736</c:v>
+                  <c:v>45781</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>45757</c:v>
+                  <c:v>45806</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>45787</c:v>
+                  <c:v>45844</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>45828</c:v>
+                  <c:v>45874</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -291,7 +294,7 @@
           <c:order val="1"/>
           <c:tx>
             <c:strRef>
-              <c:f>GANTT!$D$2</c:f>
+              <c:f>GANTT!$C$2</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -310,6 +313,64 @@
             <a:effectLst/>
           </c:spPr>
           <c:invertIfNegative val="0"/>
+          <c:dLbls>
+            <c:spPr>
+              <a:noFill/>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:txPr>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+                <a:spAutoFit/>
+              </a:bodyPr>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="75000"/>
+                        <a:lumOff val="25000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:endParaRPr lang="pt-PT"/>
+              </a:p>
+            </c:txPr>
+            <c:dLblPos val="ctr"/>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="1"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:showBubbleSize val="0"/>
+            <c:showLeaderLines val="0"/>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                <c15:showLeaderLines val="1"/>
+                <c15:leaderLines>
+                  <c:spPr>
+                    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+                      <a:solidFill>
+                        <a:schemeClr val="tx1">
+                          <a:lumMod val="35000"/>
+                          <a:lumOff val="65000"/>
+                        </a:schemeClr>
+                      </a:solidFill>
+                      <a:round/>
+                    </a:ln>
+                    <a:effectLst/>
+                  </c:spPr>
+                </c15:leaderLines>
+              </c:ext>
+            </c:extLst>
+          </c:dLbls>
           <c:cat>
             <c:strRef>
               <c:f>GANTT!$A$3:$A$10</c:f>
@@ -322,19 +383,19 @@
                   <c:v>Planeamento da arquitetura</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>Conversão dos dados de entrada para o padrão ITC 2019</c:v>
+                  <c:v>Implementação do interpretador dos dados ITC 2019</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>Implementação do interpretador dos dados ITC 2019</c:v>
+                  <c:v>Implementação da base de dados</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>Implementação da base de dados</c:v>
+                  <c:v>Implementação do simulated annealing</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>Implementação do simulated annealing</c:v>
+                  <c:v>Implementação da interface gráfica</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>Implementação da interface gráfica</c:v>
+                  <c:v>Correção de erros</c:v>
                 </c:pt>
                 <c:pt idx="7">
                   <c:v>Avaliação e correção da aplicação</c:v>
@@ -344,7 +405,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>GANTT!$D$3:$D$10</c:f>
+              <c:f>GANTT!$C$3:$C$10</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="8"/>
@@ -352,25 +413,25 @@
                   <c:v>213</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>7</c:v>
+                  <c:v>28</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>7</c:v>
+                  <c:v>21</c:v>
                 </c:pt>
                 <c:pt idx="3">
                   <c:v>21</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>21</c:v>
+                  <c:v>28</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>28</c:v>
+                  <c:v>41</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>41</c:v>
+                  <c:v>32</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>73</c:v>
+                  <c:v>56</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -423,7 +484,7 @@
           <a:lstStyle/>
           <a:p>
             <a:pPr>
-              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:defRPr sz="1100" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
                 <a:solidFill>
                   <a:schemeClr val="tx1">
                     <a:lumMod val="65000"/>
@@ -500,7 +561,7 @@
           <a:lstStyle/>
           <a:p>
             <a:pPr>
-              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
                 <a:ln>
                   <a:noFill/>
                 </a:ln>
@@ -659,7 +720,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{4C7FD7FC-901E-495B-B613-AB65D10B551C}" type="CELLRANGE">
+                    <a:fld id="{E4DDA556-25C0-49C7-BFFB-C2AB31E3CB2A}" type="CELLRANGE">
                       <a:rPr lang="pt-PT"/>
                       <a:pPr/>
                       <a:t>[INTERVALODACÉLULA]</a:t>
@@ -692,7 +753,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{16B83809-4D41-45B0-B1A7-795B9966D3D3}" type="CELLRANGE">
+                    <a:fld id="{C7797948-CBD2-4782-82F5-6CCE8CBD89B3}" type="CELLRANGE">
                       <a:rPr lang="pt-PT"/>
                       <a:pPr/>
                       <a:t>[INTERVALODACÉLULA]</a:t>
@@ -725,7 +786,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{8A1A5C0A-6A45-4159-A770-6A6A89E17A0E}" type="CELLRANGE">
+                    <a:fld id="{CA697493-1675-4FFF-BF9F-434126C16D41}" type="CELLRANGE">
                       <a:rPr lang="pt-PT"/>
                       <a:pPr/>
                       <a:t>[INTERVALODACÉLULA]</a:t>
@@ -758,7 +819,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{8D3766C9-A2F9-4B57-973D-EF66C8B3F037}" type="CELLRANGE">
+                    <a:fld id="{7FABCB2C-159E-4D63-952A-173C22F2BC95}" type="CELLRANGE">
                       <a:rPr lang="pt-PT"/>
                       <a:pPr/>
                       <a:t>[INTERVALODACÉLULA]</a:t>
@@ -791,7 +852,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{6F554FF5-A235-4E5F-8EC3-F6FB60283B4A}" type="CELLRANGE">
+                    <a:fld id="{2F98C358-5D6F-4FE5-8B50-455E8C1D9112}" type="CELLRANGE">
                       <a:rPr lang="pt-PT"/>
                       <a:pPr/>
                       <a:t>[INTERVALODACÉLULA]</a:t>
@@ -824,7 +885,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{180499CC-8A71-4089-ADA2-B9B026E4C3E9}" type="CELLRANGE">
+                    <a:fld id="{063AF7DE-04F7-4325-8BA5-97E68B85B40A}" type="CELLRANGE">
                       <a:rPr lang="pt-PT"/>
                       <a:pPr/>
                       <a:t>[INTERVALODACÉLULA]</a:t>
@@ -857,7 +918,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{35AF636C-1C9B-44AC-AF2A-39171CBCAABE}" type="CELLRANGE">
+                    <a:fld id="{8DB4ACD1-D7CF-4584-8FA1-0D6192A1AE78}" type="CELLRANGE">
                       <a:rPr lang="pt-PT"/>
                       <a:pPr/>
                       <a:t>[INTERVALODACÉLULA]</a:t>
@@ -890,7 +951,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{DB819A59-A9DC-45D3-B4FD-935645DDAAAC}" type="CELLRANGE">
+                    <a:fld id="{1034450C-21B4-4796-A582-B10F71F4DA16}" type="CELLRANGE">
                       <a:rPr lang="pt-PT"/>
                       <a:pPr/>
                       <a:t>[INTERVALODACÉLULA]</a:t>
@@ -923,7 +984,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{7A49A243-0C2F-4FFE-A8AB-D1D7BD3C4535}" type="CELLRANGE">
+                    <a:fld id="{6ED15937-E94A-4581-9B08-10DD2BFDFC54}" type="CELLRANGE">
                       <a:rPr lang="pt-PT"/>
                       <a:pPr/>
                       <a:t>[INTERVALODACÉLULA]</a:t>
@@ -956,7 +1017,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{BEBEEC8E-3C68-427C-8946-DDA8FCE8B035}" type="CELLRANGE">
+                    <a:fld id="{384BDE51-88C5-4EA2-BA6E-16F3245883B0}" type="CELLRANGE">
                       <a:rPr lang="pt-PT"/>
                       <a:pPr/>
                       <a:t>[INTERVALODACÉLULA]</a:t>
@@ -989,7 +1050,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{7C043B7E-837E-49AE-B272-08A27E6EFC03}" type="CELLRANGE">
+                    <a:fld id="{332D1287-F31A-4C7D-BB83-DC75106A575F}" type="CELLRANGE">
                       <a:rPr lang="pt-PT"/>
                       <a:pPr/>
                       <a:t>[INTERVALODACÉLULA]</a:t>
@@ -1022,7 +1083,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{7D1247E9-C7D1-431D-A655-3218C3089820}" type="CELLRANGE">
+                    <a:fld id="{F7C9F380-7915-4884-BD07-8F6BB1FDA773}" type="CELLRANGE">
                       <a:rPr lang="pt-PT"/>
                       <a:pPr/>
                       <a:t>[INTERVALODACÉLULA]</a:t>
@@ -1055,7 +1116,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{A0E6D1D0-AC34-46BA-93B9-9B0A751F2795}" type="CELLRANGE">
+                    <a:fld id="{7F78FC5F-EA73-4E01-868C-C7D2C93D0E27}" type="CELLRANGE">
                       <a:rPr lang="pt-PT"/>
                       <a:pPr/>
                       <a:t>[INTERVALODACÉLULA]</a:t>
@@ -1088,7 +1149,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{CA2CF1D4-4290-44E4-AE8D-61890CDA4A93}" type="CELLRANGE">
+                    <a:fld id="{5CC292A7-98EF-40F4-9578-4945F367DCD5}" type="CELLRANGE">
                       <a:rPr lang="pt-PT"/>
                       <a:pPr/>
                       <a:t>[INTERVALODACÉLULA]</a:t>
@@ -1121,7 +1182,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{06532B60-726B-47CE-93B2-B84D41F1AFAB}" type="CELLRANGE">
+                    <a:fld id="{33039EC4-6901-4B09-AC2C-37095D1917E6}" type="CELLRANGE">
                       <a:rPr lang="pt-PT"/>
                       <a:pPr/>
                       <a:t>[INTERVALODACÉLULA]</a:t>
@@ -1154,7 +1215,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{8E5257A3-A761-4DEE-8EC7-A239488A7EA3}" type="CELLRANGE">
+                    <a:fld id="{34A6C260-F512-4CE6-B486-94193C515F4E}" type="CELLRANGE">
                       <a:rPr lang="pt-PT"/>
                       <a:pPr/>
                       <a:t>[INTERVALODACÉLULA]</a:t>
@@ -1187,7 +1248,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{FAE214F6-788A-4020-A5C7-BD79D5D29688}" type="CELLRANGE">
+                    <a:fld id="{1EDE5214-D09E-43DA-B304-BFFD5A149D31}" type="CELLRANGE">
                       <a:rPr lang="pt-PT"/>
                       <a:pPr/>
                       <a:t>[INTERVALODACÉLULA]</a:t>
@@ -1220,7 +1281,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{53451286-C5FB-4B34-BE0F-7E4325DC4D13}" type="CELLRANGE">
+                    <a:fld id="{EA8E8D9D-91AF-422E-9ECC-1155A98BCD05}" type="CELLRANGE">
                       <a:rPr lang="pt-PT"/>
                       <a:pPr/>
                       <a:t>[INTERVALODACÉLULA]</a:t>
@@ -1253,7 +1314,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{4FEE6517-CFD8-48E6-9B11-E39E7CAFDB4F}" type="CELLRANGE">
+                    <a:fld id="{1E557C4F-82B3-4FCD-8018-F3864A3D6FAE}" type="CELLRANGE">
                       <a:rPr lang="pt-PT"/>
                       <a:pPr/>
                       <a:t>[INTERVALODACÉLULA]</a:t>
@@ -1286,7 +1347,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{5156A5FD-1FC4-475D-8EB9-DB0206378B83}" type="CELLRANGE">
+                    <a:fld id="{2534F68D-242B-4841-BE1B-B86677DA29A6}" type="CELLRANGE">
                       <a:rPr lang="pt-PT"/>
                       <a:pPr/>
                       <a:t>[INTERVALODACÉLULA]</a:t>
@@ -1319,7 +1380,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{65C33C34-3371-4FCB-970E-00E7FA3B82CD}" type="CELLRANGE">
+                    <a:fld id="{648E9DE5-AC10-4E71-9E25-496CB9B2FA5B}" type="CELLRANGE">
                       <a:rPr lang="pt-PT"/>
                       <a:pPr/>
                       <a:t>[INTERVALODACÉLULA]</a:t>
@@ -1352,7 +1413,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{227DB3BA-0A8C-47E7-AC70-67117EDAB765}" type="CELLRANGE">
+                    <a:fld id="{8D6BF847-7EF5-454C-90A9-96315032D887}" type="CELLRANGE">
                       <a:rPr lang="pt-PT"/>
                       <a:pPr/>
                       <a:t>[INTERVALODACÉLULA]</a:t>
@@ -1385,7 +1446,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{85BC8113-FEB3-4F49-A64A-7EC6715D7E0D}" type="CELLRANGE">
+                    <a:fld id="{95019767-DAA1-4EC4-B77C-16CCAE4C7E92}" type="CELLRANGE">
                       <a:rPr lang="pt-PT"/>
                       <a:pPr/>
                       <a:t>[INTERVALODACÉLULA]</a:t>
@@ -1418,7 +1479,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{18AB1DBE-5D9B-4943-9614-B8549A729B35}" type="CELLRANGE">
+                    <a:fld id="{B056264F-7E05-4904-BBF4-46DD48595A4A}" type="CELLRANGE">
                       <a:rPr lang="pt-PT"/>
                       <a:pPr/>
                       <a:t>[INTERVALODACÉLULA]</a:t>
@@ -2913,15 +2974,15 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>476249</xdr:colOff>
+      <xdr:colOff>523874</xdr:colOff>
       <xdr:row>10</xdr:row>
-      <xdr:rowOff>166687</xdr:rowOff>
+      <xdr:rowOff>138111</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>9</xdr:col>
-      <xdr:colOff>114300</xdr:colOff>
-      <xdr:row>24</xdr:row>
-      <xdr:rowOff>76200</xdr:rowOff>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>104775</xdr:colOff>
+      <xdr:row>32</xdr:row>
+      <xdr:rowOff>180974</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -3292,195 +3353,193 @@
   <cols>
     <col min="1" max="1" width="51" style="1" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="13.140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="11.140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="13.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="18" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="5" width="18" style="1" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="10.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A1" s="7" t="s">
+      <c r="A1" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="B1" s="7"/>
-      <c r="C1" s="7"/>
-      <c r="D1" s="7"/>
-      <c r="E1" s="7"/>
+      <c r="B1" s="8"/>
+      <c r="C1" s="8"/>
+      <c r="D1" s="8"/>
+      <c r="E1" s="8"/>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A2" s="1" t="s">
+      <c r="A2" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B2" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="C2" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="D2" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="E2" s="6" t="s">
         <v>10</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="E2" s="1" t="s">
-        <v>13</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A3" s="4" t="s">
+      <c r="A3" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="B3" s="2">
+      <c r="B3" s="4">
         <v>45717</v>
       </c>
-      <c r="C3" s="2">
+      <c r="C3" s="6">
+        <v>213</v>
+      </c>
+      <c r="D3" s="7">
+        <f t="shared" ref="D3:D10" si="0">C3/7</f>
+        <v>30.428571428571427</v>
+      </c>
+      <c r="E3" s="4">
+        <f>B3+C3</f>
         <v>45930</v>
       </c>
-      <c r="D3" s="1">
-        <f>C3-B3</f>
-        <v>213</v>
-      </c>
-      <c r="E3" s="5">
-        <f>D3/7</f>
-        <v>30.428571428571427</v>
-      </c>
-      <c r="G3" s="6"/>
+      <c r="G3" s="4"/>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A4" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="B4" s="2">
+      <c r="A4" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="B4" s="4">
         <v>45717</v>
       </c>
-      <c r="C4" s="2">
-        <v>45724</v>
-      </c>
-      <c r="D4" s="1">
-        <f>C4-B4</f>
-        <v>7</v>
-      </c>
-      <c r="E4" s="5">
-        <f>D4/7</f>
-        <v>1</v>
-      </c>
-      <c r="G4" s="6"/>
+      <c r="C4" s="6">
+        <v>28</v>
+      </c>
+      <c r="D4" s="7">
+        <f t="shared" si="0"/>
+        <v>4</v>
+      </c>
+      <c r="E4" s="4">
+        <f t="shared" ref="E4:E9" si="1">B4+C4</f>
+        <v>45745</v>
+      </c>
+      <c r="G4" s="4"/>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A5" s="4" t="s">
+      <c r="A5" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="B5" s="2">
-        <v>45717</v>
-      </c>
-      <c r="C5" s="2">
-        <v>45724</v>
-      </c>
-      <c r="D5" s="1">
-        <f t="shared" ref="D5" si="0">C5-B5</f>
-        <v>7</v>
-      </c>
-      <c r="E5" s="5">
-        <f t="shared" ref="E5:E10" si="1">D5/7</f>
-        <v>1</v>
-      </c>
-      <c r="G5" s="6"/>
+      <c r="B5" s="4">
+        <v>45745</v>
+      </c>
+      <c r="C5" s="6">
+        <v>21</v>
+      </c>
+      <c r="D5" s="7">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+      <c r="E5" s="4">
+        <f t="shared" si="1"/>
+        <v>45766</v>
+      </c>
+      <c r="G5" s="4"/>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A6" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="B6" s="2">
-        <v>45722</v>
-      </c>
-      <c r="C6" s="2">
-        <v>45743</v>
-      </c>
-      <c r="D6" s="1">
-        <f>C6-B6</f>
+      <c r="A6" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="B6" s="4">
+        <v>45763</v>
+      </c>
+      <c r="C6" s="6">
         <v>21</v>
       </c>
-      <c r="E6" s="5">
+      <c r="D6" s="7">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+      <c r="E6" s="4">
         <f t="shared" si="1"/>
-        <v>3</v>
-      </c>
-      <c r="G6" s="6"/>
+        <v>45784</v>
+      </c>
+      <c r="G6" s="4"/>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A7" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="B7" s="2">
-        <v>45736</v>
-      </c>
-      <c r="C7" s="2">
-        <v>45757</v>
-      </c>
-      <c r="D7" s="1">
-        <f>C7-B7</f>
-        <v>21</v>
-      </c>
-      <c r="E7" s="5">
+      <c r="A7" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="B7" s="4">
+        <v>45781</v>
+      </c>
+      <c r="C7" s="6">
+        <v>28</v>
+      </c>
+      <c r="D7" s="7">
+        <f t="shared" si="0"/>
+        <v>4</v>
+      </c>
+      <c r="E7" s="4">
         <f t="shared" si="1"/>
-        <v>3</v>
-      </c>
-      <c r="G7" s="6"/>
+        <v>45809</v>
+      </c>
+      <c r="G7" s="4"/>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A8" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="B8" s="2">
-        <v>45757</v>
-      </c>
-      <c r="C8" s="2">
-        <v>45785</v>
-      </c>
-      <c r="D8" s="1">
-        <f>C8-B8</f>
-        <v>28</v>
-      </c>
-      <c r="E8" s="5">
+      <c r="A8" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="B8" s="4">
+        <v>45806</v>
+      </c>
+      <c r="C8" s="6">
+        <v>41</v>
+      </c>
+      <c r="D8" s="7">
+        <f t="shared" si="0"/>
+        <v>5.8571428571428568</v>
+      </c>
+      <c r="E8" s="4">
         <f t="shared" si="1"/>
-        <v>4</v>
-      </c>
-      <c r="G8" s="6"/>
+        <v>45847</v>
+      </c>
+      <c r="G8" s="4"/>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A9" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="B9" s="2">
-        <v>45787</v>
-      </c>
-      <c r="C9" s="2">
-        <v>45828</v>
-      </c>
-      <c r="D9" s="1">
-        <f>C9-B9</f>
-        <v>41</v>
-      </c>
-      <c r="E9" s="5">
+      <c r="A9" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="B9" s="4">
+        <v>45844</v>
+      </c>
+      <c r="C9" s="6">
+        <v>32</v>
+      </c>
+      <c r="D9" s="7">
+        <f t="shared" si="0"/>
+        <v>4.5714285714285712</v>
+      </c>
+      <c r="E9" s="4">
         <f t="shared" si="1"/>
-        <v>5.8571428571428568</v>
-      </c>
-      <c r="G9" s="6"/>
+        <v>45876</v>
+      </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A10" s="4" t="s">
+      <c r="A10" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="B10" s="2">
-        <v>45828</v>
-      </c>
-      <c r="C10" s="2">
-        <v>45901</v>
-      </c>
-      <c r="D10" s="1">
-        <f>C10-B10</f>
-        <v>73</v>
-      </c>
-      <c r="E10" s="5">
-        <f t="shared" si="1"/>
-        <v>10.428571428571429</v>
+      <c r="B10" s="4">
+        <v>45874</v>
+      </c>
+      <c r="C10" s="6">
+        <v>56</v>
+      </c>
+      <c r="D10" s="7">
+        <f t="shared" si="0"/>
+        <v>8</v>
+      </c>
+      <c r="E10" s="4">
+        <f>B10+C10</f>
+        <v>45930</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Correction of somes images and Gantt diagram. Correction of references to listings.
</commit_message>
<xml_diff>
--- a/diagramas/diagrama_Gantt.xlsx
+++ b/diagramas/diagrama_Gantt.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Ricardo\Desktop\Tese_mestrado\diagramas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8FBB4082-AD08-4265-A554-750B0CC751D4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D5E52A1C-C719-4FB8-BD9E-B6CC89301FDC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{9E5D4881-DCE1-478A-8E87-A90D197304B3}"/>
   </bookViews>
@@ -132,7 +132,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -147,9 +147,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
@@ -158,6 +155,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -480,11 +481,11 @@
           <a:effectLst/>
         </c:spPr>
         <c:txPr>
-          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" wrap="square" anchor="ctr" anchorCtr="1"/>
           <a:lstStyle/>
           <a:p>
             <a:pPr>
-              <a:defRPr sz="1100" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:defRPr sz="1600" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
                 <a:solidFill>
                   <a:schemeClr val="tx1">
                     <a:lumMod val="65000"/>
@@ -561,7 +562,7 @@
           <a:lstStyle/>
           <a:p>
             <a:pPr>
-              <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
                 <a:ln>
                   <a:noFill/>
                 </a:ln>
@@ -608,12 +609,7 @@
       <a:schemeClr val="bg1"/>
     </a:solidFill>
     <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-      <a:solidFill>
-        <a:schemeClr val="tx1">
-          <a:lumMod val="15000"/>
-          <a:lumOff val="85000"/>
-        </a:schemeClr>
-      </a:solidFill>
+      <a:noFill/>
       <a:round/>
     </a:ln>
     <a:effectLst/>
@@ -720,7 +716,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{E4DDA556-25C0-49C7-BFFB-C2AB31E3CB2A}" type="CELLRANGE">
+                    <a:fld id="{45374623-F09F-4C67-8103-903C3D888C79}" type="CELLRANGE">
                       <a:rPr lang="pt-PT"/>
                       <a:pPr/>
                       <a:t>[INTERVALODACÉLULA]</a:t>
@@ -753,7 +749,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{C7797948-CBD2-4782-82F5-6CCE8CBD89B3}" type="CELLRANGE">
+                    <a:fld id="{D0F6DBD7-AA1A-4CC0-AC30-BE6A1D8281DE}" type="CELLRANGE">
                       <a:rPr lang="pt-PT"/>
                       <a:pPr/>
                       <a:t>[INTERVALODACÉLULA]</a:t>
@@ -772,6 +768,7 @@
               <c:extLst>
                 <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
                   <c15:dlblFieldTable/>
+                  <c15:xForSave val="1"/>
                   <c15:showDataLabelsRange val="1"/>
                 </c:ext>
                 <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
@@ -786,7 +783,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{CA697493-1675-4FFF-BF9F-434126C16D41}" type="CELLRANGE">
+                    <a:fld id="{42DE85B0-6F9B-4214-AA02-B8006A9E288D}" type="CELLRANGE">
                       <a:rPr lang="pt-PT"/>
                       <a:pPr/>
                       <a:t>[INTERVALODACÉLULA]</a:t>
@@ -805,6 +802,7 @@
               <c:extLst>
                 <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
                   <c15:dlblFieldTable/>
+                  <c15:xForSave val="1"/>
                   <c15:showDataLabelsRange val="1"/>
                 </c:ext>
                 <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
@@ -819,7 +817,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{7FABCB2C-159E-4D63-952A-173C22F2BC95}" type="CELLRANGE">
+                    <a:fld id="{B5016827-919C-4DA1-88DE-13915240B51E}" type="CELLRANGE">
                       <a:rPr lang="pt-PT"/>
                       <a:pPr/>
                       <a:t>[INTERVALODACÉLULA]</a:t>
@@ -838,6 +836,7 @@
               <c:extLst>
                 <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
                   <c15:dlblFieldTable/>
+                  <c15:xForSave val="1"/>
                   <c15:showDataLabelsRange val="1"/>
                 </c:ext>
                 <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
@@ -852,7 +851,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{2F98C358-5D6F-4FE5-8B50-455E8C1D9112}" type="CELLRANGE">
+                    <a:fld id="{013D2650-57B2-419C-B8C5-FE39A77E39DF}" type="CELLRANGE">
                       <a:rPr lang="pt-PT"/>
                       <a:pPr/>
                       <a:t>[INTERVALODACÉLULA]</a:t>
@@ -871,6 +870,7 @@
               <c:extLst>
                 <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
                   <c15:dlblFieldTable/>
+                  <c15:xForSave val="1"/>
                   <c15:showDataLabelsRange val="1"/>
                 </c:ext>
                 <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
@@ -885,7 +885,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{063AF7DE-04F7-4325-8BA5-97E68B85B40A}" type="CELLRANGE">
+                    <a:fld id="{360E8993-B033-48B0-BFFB-38EC48652099}" type="CELLRANGE">
                       <a:rPr lang="pt-PT"/>
                       <a:pPr/>
                       <a:t>[INTERVALODACÉLULA]</a:t>
@@ -904,6 +904,7 @@
               <c:extLst>
                 <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
                   <c15:dlblFieldTable/>
+                  <c15:xForSave val="1"/>
                   <c15:showDataLabelsRange val="1"/>
                 </c:ext>
                 <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
@@ -918,7 +919,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{8DB4ACD1-D7CF-4584-8FA1-0D6192A1AE78}" type="CELLRANGE">
+                    <a:fld id="{7CDE4CB1-325D-4F23-965B-4F6DA3693870}" type="CELLRANGE">
                       <a:rPr lang="pt-PT"/>
                       <a:pPr/>
                       <a:t>[INTERVALODACÉLULA]</a:t>
@@ -937,6 +938,7 @@
               <c:extLst>
                 <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
                   <c15:dlblFieldTable/>
+                  <c15:xForSave val="1"/>
                   <c15:showDataLabelsRange val="1"/>
                 </c:ext>
                 <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
@@ -951,7 +953,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{1034450C-21B4-4796-A582-B10F71F4DA16}" type="CELLRANGE">
+                    <a:fld id="{2325D08B-BE83-43D1-A791-27B297D8C204}" type="CELLRANGE">
                       <a:rPr lang="pt-PT"/>
                       <a:pPr/>
                       <a:t>[INTERVALODACÉLULA]</a:t>
@@ -970,6 +972,7 @@
               <c:extLst>
                 <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
                   <c15:dlblFieldTable/>
+                  <c15:xForSave val="1"/>
                   <c15:showDataLabelsRange val="1"/>
                 </c:ext>
                 <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
@@ -984,7 +987,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{6ED15937-E94A-4581-9B08-10DD2BFDFC54}" type="CELLRANGE">
+                    <a:fld id="{70F23ED9-417D-447D-924C-217D323F4F69}" type="CELLRANGE">
                       <a:rPr lang="pt-PT"/>
                       <a:pPr/>
                       <a:t>[INTERVALODACÉLULA]</a:t>
@@ -1003,6 +1006,7 @@
               <c:extLst>
                 <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
                   <c15:dlblFieldTable/>
+                  <c15:xForSave val="1"/>
                   <c15:showDataLabelsRange val="1"/>
                 </c:ext>
                 <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
@@ -1017,7 +1021,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{384BDE51-88C5-4EA2-BA6E-16F3245883B0}" type="CELLRANGE">
+                    <a:fld id="{86E122AC-FBF8-4E27-902D-A008E1EDDB3F}" type="CELLRANGE">
                       <a:rPr lang="pt-PT"/>
                       <a:pPr/>
                       <a:t>[INTERVALODACÉLULA]</a:t>
@@ -1036,6 +1040,7 @@
               <c:extLst>
                 <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
                   <c15:dlblFieldTable/>
+                  <c15:xForSave val="1"/>
                   <c15:showDataLabelsRange val="1"/>
                 </c:ext>
                 <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
@@ -1050,7 +1055,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{332D1287-F31A-4C7D-BB83-DC75106A575F}" type="CELLRANGE">
+                    <a:fld id="{ED12E982-AA12-4094-AF97-7C57F74366A5}" type="CELLRANGE">
                       <a:rPr lang="pt-PT"/>
                       <a:pPr/>
                       <a:t>[INTERVALODACÉLULA]</a:t>
@@ -1069,6 +1074,7 @@
               <c:extLst>
                 <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
                   <c15:dlblFieldTable/>
+                  <c15:xForSave val="1"/>
                   <c15:showDataLabelsRange val="1"/>
                 </c:ext>
                 <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
@@ -1083,7 +1089,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{F7C9F380-7915-4884-BD07-8F6BB1FDA773}" type="CELLRANGE">
+                    <a:fld id="{98AB568F-3499-4FAB-96A7-5CD524658746}" type="CELLRANGE">
                       <a:rPr lang="pt-PT"/>
                       <a:pPr/>
                       <a:t>[INTERVALODACÉLULA]</a:t>
@@ -1102,6 +1108,7 @@
               <c:extLst>
                 <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
                   <c15:dlblFieldTable/>
+                  <c15:xForSave val="1"/>
                   <c15:showDataLabelsRange val="1"/>
                 </c:ext>
                 <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
@@ -1116,7 +1123,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{7F78FC5F-EA73-4E01-868C-C7D2C93D0E27}" type="CELLRANGE">
+                    <a:fld id="{3FADBACF-0579-42E5-9E25-0FF0BC52D069}" type="CELLRANGE">
                       <a:rPr lang="pt-PT"/>
                       <a:pPr/>
                       <a:t>[INTERVALODACÉLULA]</a:t>
@@ -1135,6 +1142,7 @@
               <c:extLst>
                 <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
                   <c15:dlblFieldTable/>
+                  <c15:xForSave val="1"/>
                   <c15:showDataLabelsRange val="1"/>
                 </c:ext>
                 <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
@@ -1149,7 +1157,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{5CC292A7-98EF-40F4-9578-4945F367DCD5}" type="CELLRANGE">
+                    <a:fld id="{BB16168A-3076-4102-8222-7EDD452E0D5E}" type="CELLRANGE">
                       <a:rPr lang="pt-PT"/>
                       <a:pPr/>
                       <a:t>[INTERVALODACÉLULA]</a:t>
@@ -1168,6 +1176,7 @@
               <c:extLst>
                 <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
                   <c15:dlblFieldTable/>
+                  <c15:xForSave val="1"/>
                   <c15:showDataLabelsRange val="1"/>
                 </c:ext>
                 <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
@@ -1182,7 +1191,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{33039EC4-6901-4B09-AC2C-37095D1917E6}" type="CELLRANGE">
+                    <a:fld id="{423C03FE-2670-4DE1-BB00-F77171A9A291}" type="CELLRANGE">
                       <a:rPr lang="pt-PT"/>
                       <a:pPr/>
                       <a:t>[INTERVALODACÉLULA]</a:t>
@@ -1201,6 +1210,7 @@
               <c:extLst>
                 <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
                   <c15:dlblFieldTable/>
+                  <c15:xForSave val="1"/>
                   <c15:showDataLabelsRange val="1"/>
                 </c:ext>
                 <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
@@ -1215,7 +1225,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{34A6C260-F512-4CE6-B486-94193C515F4E}" type="CELLRANGE">
+                    <a:fld id="{857FC275-69DF-4A53-A9D8-69E7003A99F1}" type="CELLRANGE">
                       <a:rPr lang="pt-PT"/>
                       <a:pPr/>
                       <a:t>[INTERVALODACÉLULA]</a:t>
@@ -1234,6 +1244,7 @@
               <c:extLst>
                 <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
                   <c15:dlblFieldTable/>
+                  <c15:xForSave val="1"/>
                   <c15:showDataLabelsRange val="1"/>
                 </c:ext>
                 <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
@@ -1248,7 +1259,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{1EDE5214-D09E-43DA-B304-BFFD5A149D31}" type="CELLRANGE">
+                    <a:fld id="{E175E8EB-AA28-42DB-987B-008458564390}" type="CELLRANGE">
                       <a:rPr lang="pt-PT"/>
                       <a:pPr/>
                       <a:t>[INTERVALODACÉLULA]</a:t>
@@ -1267,6 +1278,7 @@
               <c:extLst>
                 <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
                   <c15:dlblFieldTable/>
+                  <c15:xForSave val="1"/>
                   <c15:showDataLabelsRange val="1"/>
                 </c:ext>
                 <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
@@ -1281,7 +1293,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{EA8E8D9D-91AF-422E-9ECC-1155A98BCD05}" type="CELLRANGE">
+                    <a:fld id="{47623DA7-3C8A-4D83-A191-DD04AFED74B4}" type="CELLRANGE">
                       <a:rPr lang="pt-PT"/>
                       <a:pPr/>
                       <a:t>[INTERVALODACÉLULA]</a:t>
@@ -1300,6 +1312,7 @@
               <c:extLst>
                 <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
                   <c15:dlblFieldTable/>
+                  <c15:xForSave val="1"/>
                   <c15:showDataLabelsRange val="1"/>
                 </c:ext>
                 <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
@@ -1314,7 +1327,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{1E557C4F-82B3-4FCD-8018-F3864A3D6FAE}" type="CELLRANGE">
+                    <a:fld id="{B4D7DFAD-E229-4578-A881-571CE033EC46}" type="CELLRANGE">
                       <a:rPr lang="pt-PT"/>
                       <a:pPr/>
                       <a:t>[INTERVALODACÉLULA]</a:t>
@@ -1333,6 +1346,7 @@
               <c:extLst>
                 <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
                   <c15:dlblFieldTable/>
+                  <c15:xForSave val="1"/>
                   <c15:showDataLabelsRange val="1"/>
                 </c:ext>
                 <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
@@ -1347,7 +1361,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{2534F68D-242B-4841-BE1B-B86677DA29A6}" type="CELLRANGE">
+                    <a:fld id="{D6BD19EA-356D-45D5-98B7-002B5219A555}" type="CELLRANGE">
                       <a:rPr lang="pt-PT"/>
                       <a:pPr/>
                       <a:t>[INTERVALODACÉLULA]</a:t>
@@ -1366,6 +1380,7 @@
               <c:extLst>
                 <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
                   <c15:dlblFieldTable/>
+                  <c15:xForSave val="1"/>
                   <c15:showDataLabelsRange val="1"/>
                 </c:ext>
                 <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
@@ -1380,7 +1395,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{648E9DE5-AC10-4E71-9E25-496CB9B2FA5B}" type="CELLRANGE">
+                    <a:fld id="{803281E4-F411-4EF8-A0DA-AB1B16A6E33B}" type="CELLRANGE">
                       <a:rPr lang="pt-PT"/>
                       <a:pPr/>
                       <a:t>[INTERVALODACÉLULA]</a:t>
@@ -1399,6 +1414,7 @@
               <c:extLst>
                 <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
                   <c15:dlblFieldTable/>
+                  <c15:xForSave val="1"/>
                   <c15:showDataLabelsRange val="1"/>
                 </c:ext>
                 <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
@@ -1413,7 +1429,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{8D6BF847-7EF5-454C-90A9-96315032D887}" type="CELLRANGE">
+                    <a:fld id="{16FC0436-D07F-4320-A304-88D6FF14C726}" type="CELLRANGE">
                       <a:rPr lang="pt-PT"/>
                       <a:pPr/>
                       <a:t>[INTERVALODACÉLULA]</a:t>
@@ -1432,6 +1448,7 @@
               <c:extLst>
                 <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
                   <c15:dlblFieldTable/>
+                  <c15:xForSave val="1"/>
                   <c15:showDataLabelsRange val="1"/>
                 </c:ext>
                 <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
@@ -1446,7 +1463,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{95019767-DAA1-4EC4-B77C-16CCAE4C7E92}" type="CELLRANGE">
+                    <a:fld id="{6C2EC9EB-7CAF-4AA8-981A-143F702B5D72}" type="CELLRANGE">
                       <a:rPr lang="pt-PT"/>
                       <a:pPr/>
                       <a:t>[INTERVALODACÉLULA]</a:t>
@@ -1465,6 +1482,7 @@
               <c:extLst>
                 <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
                   <c15:dlblFieldTable/>
+                  <c15:xForSave val="1"/>
                   <c15:showDataLabelsRange val="1"/>
                 </c:ext>
                 <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
@@ -1479,7 +1497,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{B056264F-7E05-4904-BBF4-46DD48595A4A}" type="CELLRANGE">
+                    <a:fld id="{03A93829-41E3-4D79-A822-900642C533DC}" type="CELLRANGE">
                       <a:rPr lang="pt-PT"/>
                       <a:pPr/>
                       <a:t>[INTERVALODACÉLULA]</a:t>
@@ -1498,6 +1516,7 @@
               <c:extLst>
                 <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
                   <c15:dlblFieldTable/>
+                  <c15:xForSave val="1"/>
                   <c15:showDataLabelsRange val="1"/>
                 </c:ext>
                 <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
@@ -2974,15 +2993,15 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>523874</xdr:colOff>
-      <xdr:row>10</xdr:row>
-      <xdr:rowOff>138111</xdr:rowOff>
+      <xdr:colOff>714372</xdr:colOff>
+      <xdr:row>17</xdr:row>
+      <xdr:rowOff>81643</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>10</xdr:col>
-      <xdr:colOff>104775</xdr:colOff>
-      <xdr:row>32</xdr:row>
-      <xdr:rowOff>180974</xdr:rowOff>
+      <xdr:col>19</xdr:col>
+      <xdr:colOff>340178</xdr:colOff>
+      <xdr:row>33</xdr:row>
+      <xdr:rowOff>167367</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -3348,53 +3367,55 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5BF3AA6B-9DCA-46B7-9978-7DB82B4E0B9C}">
-  <dimension ref="A1:G10"/>
+  <dimension ref="A1:L11"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="51" style="1" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="36.7109375" style="1" customWidth="1"/>
     <col min="2" max="2" width="13.140625" style="1" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="13.7109375" style="1" bestFit="1" customWidth="1"/>
     <col min="4" max="5" width="18" style="1" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="10.7109375" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="12" customWidth="1"/>
+    <col min="12" max="12" width="12.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A1" s="8" t="s">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="B1" s="8"/>
-      <c r="C1" s="8"/>
-      <c r="D1" s="8"/>
-      <c r="E1" s="8"/>
+      <c r="B1" s="7"/>
+      <c r="C1" s="7"/>
+      <c r="D1" s="7"/>
+      <c r="E1" s="7"/>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A2" s="6" t="s">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A2" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="B2" s="6" t="s">
+      <c r="B2" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="C2" s="6" t="s">
+      <c r="C2" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="D2" s="6" t="s">
+      <c r="D2" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="E2" s="6" t="s">
+      <c r="E2" s="5" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A3" s="5" t="s">
+    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A3" s="8" t="s">
         <v>5</v>
       </c>
       <c r="B3" s="4">
         <v>45717</v>
       </c>
-      <c r="C3" s="6">
+      <c r="C3" s="5">
         <v>213</v>
       </c>
-      <c r="D3" s="7">
+      <c r="D3" s="6">
         <f t="shared" ref="D3:D10" si="0">C3/7</f>
         <v>30.428571428571427</v>
       </c>
@@ -3404,17 +3425,17 @@
       </c>
       <c r="G3" s="4"/>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A4" s="5" t="s">
+    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A4" s="8" t="s">
         <v>15</v>
       </c>
       <c r="B4" s="4">
         <v>45717</v>
       </c>
-      <c r="C4" s="6">
+      <c r="C4" s="5">
         <v>28</v>
       </c>
-      <c r="D4" s="7">
+      <c r="D4" s="6">
         <f t="shared" si="0"/>
         <v>4</v>
       </c>
@@ -3424,17 +3445,17 @@
       </c>
       <c r="G4" s="4"/>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A5" s="5" t="s">
+    <row r="5" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+      <c r="A5" s="8" t="s">
         <v>14</v>
       </c>
       <c r="B5" s="4">
         <v>45745</v>
       </c>
-      <c r="C5" s="6">
+      <c r="C5" s="5">
         <v>21</v>
       </c>
-      <c r="D5" s="7">
+      <c r="D5" s="6">
         <f t="shared" si="0"/>
         <v>3</v>
       </c>
@@ -3444,17 +3465,17 @@
       </c>
       <c r="G5" s="4"/>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A6" s="5" t="s">
+    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A6" s="8" t="s">
         <v>11</v>
       </c>
       <c r="B6" s="4">
         <v>45763</v>
       </c>
-      <c r="C6" s="6">
+      <c r="C6" s="5">
         <v>21</v>
       </c>
-      <c r="D6" s="7">
+      <c r="D6" s="6">
         <f t="shared" si="0"/>
         <v>3</v>
       </c>
@@ -3464,17 +3485,17 @@
       </c>
       <c r="G6" s="4"/>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A7" s="5" t="s">
+    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A7" s="8" t="s">
         <v>6</v>
       </c>
       <c r="B7" s="4">
         <v>45781</v>
       </c>
-      <c r="C7" s="6">
+      <c r="C7" s="5">
         <v>28</v>
       </c>
-      <c r="D7" s="7">
+      <c r="D7" s="6">
         <f t="shared" si="0"/>
         <v>4</v>
       </c>
@@ -3484,17 +3505,17 @@
       </c>
       <c r="G7" s="4"/>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A8" s="5" t="s">
+    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A8" s="8" t="s">
         <v>7</v>
       </c>
       <c r="B8" s="4">
         <v>45806</v>
       </c>
-      <c r="C8" s="6">
+      <c r="C8" s="5">
         <v>41</v>
       </c>
-      <c r="D8" s="7">
+      <c r="D8" s="6">
         <f t="shared" si="0"/>
         <v>5.8571428571428568</v>
       </c>
@@ -3504,17 +3525,17 @@
       </c>
       <c r="G8" s="4"/>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A9" s="5" t="s">
+    <row r="9" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A9" s="8" t="s">
         <v>16</v>
       </c>
       <c r="B9" s="4">
         <v>45844</v>
       </c>
-      <c r="C9" s="6">
+      <c r="C9" s="5">
         <v>32</v>
       </c>
-      <c r="D9" s="7">
+      <c r="D9" s="6">
         <f t="shared" si="0"/>
         <v>4.5714285714285712</v>
       </c>
@@ -3523,17 +3544,17 @@
         <v>45876</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A10" s="5" t="s">
+    <row r="10" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A10" s="8" t="s">
         <v>8</v>
       </c>
       <c r="B10" s="4">
         <v>45874</v>
       </c>
-      <c r="C10" s="6">
+      <c r="C10" s="5">
         <v>56</v>
       </c>
-      <c r="D10" s="7">
+      <c r="D10" s="6">
         <f t="shared" si="0"/>
         <v>8</v>
       </c>
@@ -3541,6 +3562,10 @@
         <f>B10+C10</f>
         <v>45930</v>
       </c>
+    </row>
+    <row r="11" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="K11" s="9"/>
+      <c r="L11" s="9"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>